<commit_message>
actualiza acumulados 17/06/2026 11:52
</commit_message>
<xml_diff>
--- a/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO-ARGELIA-(IED)-501_20260616_204525.xlsx
+++ b/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO-ARGELIA-(IED)-501_20260616_204525.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\COLEGIOS 3-06-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\PRUEBAS A CALIFICAR\Ya procesadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D837930-A7C5-4F8E-AA19-41D983C888D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DAA4D01-AAFF-40CF-BC84-7EE5AF2882C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resultados" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Resultados!$A$1:$AB$1</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -7162,6 +7165,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AB1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="I2:AB75">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>" "</formula>

</xml_diff>